<commit_message>
changes in ptw master and type of work
</commit_message>
<xml_diff>
--- a/public/assets/documents/excel/sample_upload/Checklist.xlsx
+++ b/public/assets/documents/excel/sample_upload/Checklist.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\xampp8.2\htdocs\NeoEHS\NeoEHS_Karam\public\assets\documents\excel\sample_upload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\projects\Ardhas\NeoEHS_Karam\public\assets\documents\excel\sample_upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CEB5CBA-E032-4A63-8C8A-F8D62446898C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="8772"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,19 +25,19 @@
     <t>SNo</t>
   </si>
   <si>
-    <t>Name</t>
-  </si>
-  <si>
     <t>Provide Safe Working Environment and Platform</t>
   </si>
   <si>
     <t>Use Proper Job Specific PPEs.</t>
   </si>
+  <si>
+    <t>Checklist</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -346,7 +347,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
@@ -358,7 +359,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -366,7 +367,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -374,7 +375,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>